<commit_message>
cleanup docs and website after recent changes
</commit_message>
<xml_diff>
--- a/docs/operation-modes.xlsx
+++ b/docs/operation-modes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rse/Work/ase/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rse/Work/ase/master/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{650D8D3E-1954-2B43-9607-C1E84958B1A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9705EEA-B6EE-DF4C-A584-3355037D355A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11060" yWindow="7040" windowWidth="28040" windowHeight="17180" xr2:uid="{10B8B807-6256-AB4F-8C12-E23F0A365D36}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$B$2:$H$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$B$2:$G$11</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -42,14 +42,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="15">
   <si>
     <t>Task Mode</t>
   </si>
   <si>
-    <t>Funnel Mode</t>
-  </si>
-  <si>
     <t>Deferred Execution</t>
   </si>
   <si>
@@ -75,9 +72,6 @@
   </si>
   <si>
     <t>X</t>
-  </si>
-  <si>
-    <t>Quick Mode</t>
   </si>
   <si>
     <t>Tenet-Driven</t>
@@ -112,6 +106,9 @@
       </rPr>
       <t>(Standard)</t>
     </r>
+  </si>
+  <si>
+    <t>Direct Mode</t>
   </si>
 </sst>
 </file>
@@ -168,7 +165,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -190,12 +187,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF368DDF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0C4171"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -290,21 +281,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -316,17 +307,14 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -677,243 +665,216 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE0BCE1A-3256-2A44-A2BA-6EC1A7EA6376}">
-  <dimension ref="B2:J16"/>
+  <dimension ref="B2:I16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.5" customWidth="1"/>
     <col min="2" max="2" width="23.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="3.6640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="3.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.83203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="4" style="1" customWidth="1"/>
-    <col min="9" max="9" width="3.5" style="1" customWidth="1"/>
-    <col min="10" max="10" width="4" customWidth="1"/>
+    <col min="6" max="7" width="4" style="1" customWidth="1"/>
+    <col min="8" max="8" width="3.5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" ht="157" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:9" ht="157" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>11</v>
-      </c>
       <c r="E2" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="J2" s="1"/>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B3" s="11" t="s">
-        <v>3</v>
+        <v>8</v>
+      </c>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B3" s="10" t="s">
+        <v>2</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3"/>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B4" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="15"/>
+      <c r="H3"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="14"/>
       <c r="D4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="14"/>
+      <c r="F4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4"/>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B5" s="10" t="s">
         <v>10</v>
-      </c>
-      <c r="E4" s="15"/>
-      <c r="F4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" s="15"/>
-      <c r="I4"/>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B5" s="11" t="s">
-        <v>12</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I5"/>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B6" s="12" t="s">
-        <v>2</v>
+        <v>9</v>
+      </c>
+      <c r="H5"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B6" s="11" t="s">
+        <v>1</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I6"/>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B7" s="12" t="s">
-        <v>5</v>
+        <v>9</v>
+      </c>
+      <c r="H6"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B7" s="11" t="s">
+        <v>4</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I7"/>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B8" s="13" t="s">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="H7"/>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B8" s="12" t="s">
+        <v>5</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="3"/>
       <c r="F8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H8" s="3"/>
-      <c r="I8"/>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B9" s="13" t="s">
-        <v>4</v>
+        <v>9</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B9" s="12" t="s">
+        <v>3</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="3"/>
       <c r="F9" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I9"/>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B10" s="14" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="H9"/>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B10" s="13" t="s">
+        <v>7</v>
       </c>
       <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
+      <c r="D10" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H10" s="3"/>
-      <c r="I10"/>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B11" s="14" t="s">
-        <v>7</v>
+      <c r="F10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10"/>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B11" s="13" t="s">
+        <v>6</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="D11" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H11" s="3"/>
-      <c r="I11"/>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="F11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="H11"/>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.2">
       <c r="C12"/>
       <c r="D12"/>
       <c r="E12"/>
       <c r="F12"/>
       <c r="G12"/>
       <c r="H12"/>
-      <c r="I12"/>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.2">
       <c r="C13"/>
       <c r="D13"/>
       <c r="E13"/>
       <c r="F13"/>
       <c r="G13"/>
       <c r="H13"/>
-      <c r="I13"/>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.2">
       <c r="C14"/>
       <c r="D14"/>
       <c r="E14"/>
       <c r="F14"/>
       <c r="G14"/>
       <c r="H14"/>
-      <c r="I14"/>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.2">
       <c r="C15"/>
       <c r="D15"/>
       <c r="E15"/>
       <c r="F15"/>
       <c r="G15"/>
       <c r="H15"/>
-      <c r="I15"/>
-    </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.2">
       <c r="C16"/>
       <c r="D16"/>
       <c r="E16"/>
       <c r="F16"/>
       <c r="G16"/>
       <c r="H16"/>
-      <c r="I16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>